<commit_message>
file naming tests complete
</commit_message>
<xml_diff>
--- a/testing/test_documents/test_register_2.xlsx
+++ b/testing/test_documents/test_register_2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cambridgeorg-my.sharepoint.com/personal/freemansmith_w_cambridgeenglish_org/Documents/Documents/Coding/python/epa-project/assets/test_registers/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cambridgeorg-my.sharepoint.com/personal/freemansmith_w_cambridgeenglish_org/Documents/Documents/Coding/python/epa-project/testing/test_documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="13_ncr:1_{C93F7102-43D8-4693-AA9A-52DB67C570BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5D41D59-6D2A-491F-AB26-E870432647F8}"/>
+  <xr:revisionPtr revIDLastSave="108" documentId="13_ncr:1_{C93F7102-43D8-4693-AA9A-52DB67C570BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDE1579D-DB82-4D08-9F06-9C75F8FC2421}"/>
   <bookViews>
-    <workbookView xWindow="26145" yWindow="-15600" windowWidth="19440" windowHeight="15000" xr2:uid="{35D4E4FF-310B-481D-90F2-EF205B6CB8C0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{35D4E4FF-310B-481D-90F2-EF205B6CB8C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="1" r:id="rId1"/>
@@ -1009,7 +1009,7 @@
         <v>20</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
@@ -5001,6 +5001,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010067E8EF0C91F44D4DB49E059C1CE9D396" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2562ec86366f66fd9495a6aeceb5bee6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5eda3a55-7787-4436-87b0-c239f96dda93" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="95db2b5860af5c3fbfe0510c0dd5fddc" ns2:_="">
     <xsd:import namespace="5eda3a55-7787-4436-87b0-c239f96dda93"/>
@@ -5198,15 +5207,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E582D512-2AB3-4D4A-B94D-63ACF495A52B}">
   <ds:schemaRefs>
@@ -5218,6 +5218,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAFCD22-1EEB-46A9-B5A6-EC079D8FA406}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{435D4061-D8E0-40AE-9068-B7974CF431D9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5233,12 +5241,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAFCD22-1EEB-46A9-B5A6-EC079D8FA406}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>